<commit_message>
removed(env, version): env replaced with docker volume mapping nad updated serde_saphyr version
</commit_message>
<xml_diff>
--- a/Database/Merch.xlsx
+++ b/Database/Merch.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="32">
   <si>
     <t>Order Id</t>
     <phoneticPr fontId="1"/>
@@ -102,6 +102,46 @@
   </si>
   <si>
     <t>Additional Notes</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>d245b4ce-6c2b-425d-aed2-10205d0ac3a4</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>HERO-2020 HOODIES</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>S</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t/>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>XL</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>brock.tomlinson@ucalgary.ca</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2509466196</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Brock</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Software</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Canada</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -406,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="6" width="8.38" customWidth="1"/>
@@ -430,6 +470,46 @@
       </c>
       <c r="F1" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2">
+        <v>36.0099983215332</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3">
+        <v>36.0099983215332</v>
       </c>
     </row>
   </sheetData>
@@ -440,7 +520,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="17" width="8.38" customWidth="1"/>
@@ -499,6 +579,56 @@
         <v>21</v>
       </c>
     </row>
+    <row r="2" spans="1:17">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2">
+        <v>72.0199966430664</v>
+      </c>
+      <c r="G2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
docs(dep): re added serde_json for tests
</commit_message>
<xml_diff>
--- a/Database/Merch.xlsx
+++ b/Database/Merch.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>Order Id</t>
     <phoneticPr fontId="1"/>
@@ -102,46 +102,6 @@
   </si>
   <si>
     <t>Additional Notes</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>d245b4ce-6c2b-425d-aed2-10205d0ac3a4</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>HERO-2020 HOODIES</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>S</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t/>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>XL</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>brock.tomlinson@ucalgary.ca</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2509466196</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Brock</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Software</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Canada</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -446,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="6" width="8.38" customWidth="1"/>
@@ -470,46 +430,6 @@
       </c>
       <c r="F1" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2">
-        <v>3</v>
-      </c>
-      <c r="E2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2">
-        <v>36.0099983215332</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3">
-        <v>36.0099983215332</v>
       </c>
     </row>
   </sheetData>
@@ -520,7 +440,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="17" width="8.38" customWidth="1"/>
@@ -579,56 +499,6 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
-      <c r="A2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F2">
-        <v>72.0199966430664</v>
-      </c>
-      <c r="G2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I2" t="s">
-        <v>25</v>
-      </c>
-      <c r="J2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O2" t="s">
-        <v>25</v>
-      </c>
-      <c r="P2" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>25</v>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>